<commit_message>
fix: XLSX upload ArrayBuffer, warnings lignes invalides, hyperliens signatures
</commit_message>
<xml_diff>
--- a/TEST.xlsx
+++ b/TEST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexcohenskalli/Documents/PERSO/Gavroch.dev/Gavroch.dev/hatmada/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2620BC22-49CE-884A-9A3E-18AB84B2E0BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ECE6F05-E2BA-6847-80B8-971E891E09FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{6748F77D-2A60-DC47-8FB3-BA892948F9D5}"/>
   </bookViews>
@@ -41,15 +41,6 @@
     <t>Cohen-Skalli</t>
   </si>
   <si>
-    <t>Alexandre</t>
-  </si>
-  <si>
-    <t>alexcoh07@gmail.com</t>
-  </si>
-  <si>
-    <t>Hatmada</t>
-  </si>
-  <si>
     <t>Prénom</t>
   </si>
   <si>
@@ -77,7 +68,16 @@
     <t>DG</t>
   </si>
   <si>
-    <t>hatmadaprospection.com</t>
+    <t>Carrefour</t>
+  </si>
+  <si>
+    <t>carrefour.com</t>
+  </si>
+  <si>
+    <t>alexcoh07gmail.com</t>
+  </si>
+  <si>
+    <t>kk</t>
   </si>
 </sst>
 </file>
@@ -488,59 +488,60 @@
   <cols>
     <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{904399F0-8935-3144-B345-779A0930DB70}"/>
+    <hyperlink ref="E2" r:id="rId1" display="raphael.c.skalli@gmail.com" xr:uid="{904399F0-8935-3144-B345-779A0930DB70}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>